<commit_message>
fix: hide empty columns and rows in new excel template
Signed-off-by: Mats Johansson <extern.mats.johansson@digg.se>
</commit_message>
<xml_diff>
--- a/document/Avstaemning_REST_API_profil_v_2_0_0_0.xlsx
+++ b/document/Avstaemning_REST_API_profil_v_2_0_0_0.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\mats\repos\rest-api-profil-lint-processor\document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6950323E-8A3E-41A5-AA53-92EF5CA6F13D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98FDF71D-4709-4F18-9EAF-1693F5E5FCBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23190" yWindow="0" windowWidth="15315" windowHeight="20985" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="1" r:id="rId1"/>
@@ -8050,6 +8050,9 @@
     <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
     </xf>
@@ -8059,16 +8062,13 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="21" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -8419,94 +8419,96 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AW49"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AW50"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" zeroHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="1" customWidth="1"/>
     <col min="2" max="13" width="10.7109375" style="2" customWidth="1"/>
-    <col min="14" max="49" width="8.7109375" style="2"/>
+    <col min="14" max="23" width="8.7109375" style="2" customWidth="1"/>
+    <col min="24" max="49" width="0" style="2" hidden="1"/>
+    <col min="50" max="16384" width="8.7109375" hidden="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:24" s="3" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="77" t="s">
+      <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="77"/>
-      <c r="C1" s="77"/>
-      <c r="D1" s="77"/>
-      <c r="E1" s="77"/>
-      <c r="F1" s="77"/>
-      <c r="G1" s="77"/>
-      <c r="H1" s="77"/>
-      <c r="I1" s="77"/>
-      <c r="J1" s="77"/>
-      <c r="K1" s="77"/>
-      <c r="L1" s="77"/>
-      <c r="M1" s="77"/>
-      <c r="N1" s="77"/>
-      <c r="O1" s="77"/>
-      <c r="P1" s="77"/>
-      <c r="Q1" s="77"/>
-      <c r="R1" s="77"/>
-      <c r="S1" s="77"/>
-      <c r="T1" s="77"/>
-      <c r="U1" s="77"/>
-      <c r="V1" s="77"/>
-      <c r="W1" s="77"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="78"/>
+      <c r="M1" s="78"/>
+      <c r="N1" s="78"/>
+      <c r="O1" s="78"/>
+      <c r="P1" s="78"/>
+      <c r="Q1" s="78"/>
+      <c r="R1" s="78"/>
+      <c r="S1" s="78"/>
+      <c r="T1" s="78"/>
+      <c r="U1" s="78"/>
+      <c r="V1" s="78"/>
+      <c r="W1" s="78"/>
     </row>
     <row r="2" spans="1:24" ht="135" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="78" t="s">
+      <c r="A2" s="79" t="s">
         <v>385</v>
       </c>
-      <c r="B2" s="78"/>
-      <c r="C2" s="78"/>
-      <c r="D2" s="78"/>
-      <c r="E2" s="78"/>
-      <c r="F2" s="78"/>
-      <c r="G2" s="78"/>
-      <c r="H2" s="78"/>
-      <c r="I2" s="78"/>
-      <c r="J2" s="78"/>
-      <c r="K2" s="78"/>
-      <c r="L2" s="78"/>
-      <c r="M2" s="78"/>
-      <c r="N2" s="78"/>
-      <c r="O2" s="79" t="s">
+      <c r="B2" s="79"/>
+      <c r="C2" s="79"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="79"/>
+      <c r="F2" s="79"/>
+      <c r="G2" s="79"/>
+      <c r="H2" s="79"/>
+      <c r="I2" s="79"/>
+      <c r="J2" s="79"/>
+      <c r="K2" s="79"/>
+      <c r="L2" s="79"/>
+      <c r="M2" s="79"/>
+      <c r="N2" s="79"/>
+      <c r="O2" s="80" t="s">
         <v>1</v>
       </c>
-      <c r="P2" s="79"/>
-      <c r="Q2" s="79"/>
-      <c r="R2" s="79"/>
-      <c r="S2" s="79"/>
-      <c r="T2" s="79"/>
-      <c r="U2" s="79"/>
+      <c r="P2" s="80"/>
+      <c r="Q2" s="80"/>
+      <c r="R2" s="80"/>
+      <c r="S2" s="80"/>
+      <c r="T2" s="80"/>
+      <c r="U2" s="80"/>
       <c r="X2" s="1"/>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A3" s="83" t="str">
+      <c r="A3" s="81" t="str">
         <f>"Kraven avser version "&amp;profilversion&amp;" av REST API profilen som i juni 2026 publicerades på https://dev.dataportal.se/rest-api-profil"</f>
         <v>Kraven avser version 2.0.0 av REST API profilen som i juni 2026 publicerades på https://dev.dataportal.se/rest-api-profil</v>
       </c>
-      <c r="B3" s="83"/>
-      <c r="C3" s="83"/>
-      <c r="D3" s="83"/>
-      <c r="E3" s="83"/>
-      <c r="F3" s="83"/>
-      <c r="G3" s="83"/>
-      <c r="H3" s="83"/>
-      <c r="I3" s="83"/>
-      <c r="J3" s="83"/>
-      <c r="K3" s="83"/>
-      <c r="L3" s="83"/>
-      <c r="M3" s="83"/>
-      <c r="N3" s="83"/>
-      <c r="O3" s="82"/>
-      <c r="P3" s="82"/>
-      <c r="Q3" s="82"/>
-      <c r="R3" s="82"/>
-      <c r="S3" s="82"/>
-      <c r="T3" s="82"/>
-      <c r="U3" s="82"/>
+      <c r="B3" s="81"/>
+      <c r="C3" s="81"/>
+      <c r="D3" s="81"/>
+      <c r="E3" s="81"/>
+      <c r="F3" s="81"/>
+      <c r="G3" s="81"/>
+      <c r="H3" s="81"/>
+      <c r="I3" s="81"/>
+      <c r="J3" s="81"/>
+      <c r="K3" s="81"/>
+      <c r="L3" s="81"/>
+      <c r="M3" s="81"/>
+      <c r="N3" s="81"/>
+      <c r="O3" s="77"/>
+      <c r="P3" s="77"/>
+      <c r="Q3" s="77"/>
+      <c r="R3" s="77"/>
+      <c r="S3" s="77"/>
+      <c r="T3" s="77"/>
+      <c r="U3" s="77"/>
       <c r="X3" s="1"/>
     </row>
     <row r="4" spans="1:24" s="6" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -8591,6 +8593,7 @@
         <v>10</v>
       </c>
     </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.25"/>
     <row r="10" spans="1:24" s="7" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>11</v>
@@ -8744,6 +8747,7 @@
         <v>10</v>
       </c>
     </row>
+    <row r="15" spans="1:24" x14ac:dyDescent="0.25"/>
     <row r="16" spans="1:24" s="17" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="str">
         <f>('Kravlista REST API profil'!$A33)</f>
@@ -8892,6 +8896,7 @@
         <v>10</v>
       </c>
     </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25"/>
     <row r="21" spans="1:13" s="17" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="str">
         <f>('Kravlista REST API profil'!$A51)</f>
@@ -9040,6 +9045,7 @@
         <v>10</v>
       </c>
     </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25"/>
     <row r="26" spans="1:13" s="17" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="17" t="str">
         <f>('Kravlista REST API profil'!$A96)</f>
@@ -9188,6 +9194,7 @@
         <v>10</v>
       </c>
     </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25"/>
     <row r="31" spans="1:13" s="17" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="17" t="str">
         <f>('Kravlista REST API profil'!$A111)</f>
@@ -10074,6 +10081,7 @@
         <v>10</v>
       </c>
     </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:W1"/>
@@ -10089,7 +10097,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:BJ423"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="15.75" zeroHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.5703125" style="19" customWidth="1"/>
     <col min="2" max="2" width="9.28515625" style="20" customWidth="1"/>
@@ -10097,9 +10105,9 @@
     <col min="4" max="4" width="12" style="20" customWidth="1"/>
     <col min="5" max="5" width="11.140625" style="21" customWidth="1"/>
     <col min="6" max="6" width="38.5703125" style="22" customWidth="1"/>
-    <col min="7" max="7" width="8.7109375" style="23"/>
-    <col min="8" max="62" width="8.7109375" style="24"/>
-    <col min="63" max="16384" width="8.7109375" style="20"/>
+    <col min="7" max="7" width="8.7109375" style="23" customWidth="1"/>
+    <col min="8" max="62" width="0" style="24" hidden="1"/>
+    <col min="63" max="16384" width="8.7109375" style="20" hidden="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:62" s="28" customFormat="1" x14ac:dyDescent="0.25">
@@ -11978,7 +11986,7 @@
       <c r="G114" s="27"/>
     </row>
     <row r="115" spans="1:7" ht="96.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A115" s="80" t="s">
+      <c r="A115" s="82" t="s">
         <v>167</v>
       </c>
       <c r="B115" s="42" t="s">
@@ -11997,7 +12005,7 @@
       <c r="G115" s="27"/>
     </row>
     <row r="116" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A116" s="80"/>
+      <c r="A116" s="82"/>
       <c r="B116" s="63" t="s">
         <v>234</v>
       </c>
@@ -12509,7 +12517,7 @@
       <c r="G147" s="27"/>
     </row>
     <row r="148" spans="1:7" ht="37.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A148" s="81" t="s">
+      <c r="A148" s="83" t="s">
         <v>294</v>
       </c>
       <c r="B148" s="42" t="s">
@@ -12528,7 +12536,7 @@
       <c r="G148" s="27"/>
     </row>
     <row r="149" spans="1:7" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A149" s="81"/>
+      <c r="A149" s="83"/>
       <c r="B149" s="30" t="s">
         <v>297</v>
       </c>
@@ -12545,7 +12553,7 @@
       <c r="G149" s="27"/>
     </row>
     <row r="150" spans="1:7" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A150" s="81"/>
+      <c r="A150" s="83"/>
       <c r="B150" s="30" t="s">
         <v>299</v>
       </c>
@@ -12562,7 +12570,7 @@
       <c r="G150" s="27"/>
     </row>
     <row r="151" spans="1:7" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A151" s="81"/>
+      <c r="A151" s="83"/>
       <c r="B151" s="30" t="s">
         <v>301</v>
       </c>
@@ -12579,7 +12587,7 @@
       <c r="G151" s="27"/>
     </row>
     <row r="152" spans="1:7" ht="63" x14ac:dyDescent="0.25">
-      <c r="A152" s="81"/>
+      <c r="A152" s="83"/>
       <c r="B152" s="30" t="s">
         <v>303</v>
       </c>
@@ -12596,7 +12604,7 @@
       <c r="G152" s="27"/>
     </row>
     <row r="153" spans="1:7" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A153" s="81"/>
+      <c r="A153" s="83"/>
       <c r="B153" s="38" t="s">
         <v>305</v>
       </c>
@@ -13284,1363 +13292,1363 @@
       <c r="F196" s="23"/>
       <c r="G196" s="23"/>
     </row>
-    <row r="197" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A197" s="75"/>
       <c r="E197" s="76"/>
       <c r="F197" s="23"/>
       <c r="G197" s="23"/>
     </row>
-    <row r="198" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A198" s="75"/>
       <c r="E198" s="76"/>
       <c r="F198" s="23"/>
       <c r="G198" s="23"/>
     </row>
-    <row r="199" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A199" s="75"/>
       <c r="E199" s="76"/>
       <c r="F199" s="23"/>
       <c r="G199" s="23"/>
     </row>
-    <row r="200" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A200" s="75"/>
       <c r="E200" s="76"/>
       <c r="F200" s="23"/>
       <c r="G200" s="23"/>
     </row>
-    <row r="201" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A201" s="75"/>
       <c r="E201" s="76"/>
       <c r="F201" s="23"/>
       <c r="G201" s="23"/>
     </row>
-    <row r="202" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A202" s="75"/>
       <c r="E202" s="76"/>
       <c r="F202" s="23"/>
       <c r="G202" s="23"/>
     </row>
-    <row r="203" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A203" s="75"/>
       <c r="E203" s="76"/>
       <c r="F203" s="23"/>
       <c r="G203" s="23"/>
     </row>
-    <row r="204" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A204" s="75"/>
       <c r="E204" s="76"/>
       <c r="F204" s="23"/>
       <c r="G204" s="23"/>
     </row>
-    <row r="205" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A205" s="75"/>
       <c r="E205" s="76"/>
       <c r="F205" s="23"/>
       <c r="G205" s="23"/>
     </row>
-    <row r="206" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A206" s="75"/>
       <c r="E206" s="76"/>
       <c r="F206" s="23"/>
       <c r="G206" s="23"/>
     </row>
-    <row r="207" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A207" s="75"/>
       <c r="E207" s="76"/>
       <c r="F207" s="23"/>
       <c r="G207" s="23"/>
     </row>
-    <row r="208" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A208" s="75"/>
       <c r="E208" s="76"/>
       <c r="F208" s="23"/>
       <c r="G208" s="23"/>
     </row>
-    <row r="209" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A209" s="75"/>
       <c r="E209" s="76"/>
       <c r="F209" s="23"/>
       <c r="G209" s="23"/>
     </row>
-    <row r="210" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A210" s="75"/>
       <c r="E210" s="76"/>
       <c r="F210" s="23"/>
       <c r="G210" s="23"/>
     </row>
-    <row r="211" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A211" s="75"/>
       <c r="E211" s="76"/>
       <c r="F211" s="23"/>
       <c r="G211" s="23"/>
     </row>
-    <row r="212" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A212" s="75"/>
       <c r="E212" s="76"/>
       <c r="F212" s="23"/>
       <c r="G212" s="23"/>
     </row>
-    <row r="213" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A213" s="75"/>
       <c r="E213" s="76"/>
       <c r="F213" s="23"/>
       <c r="G213" s="23"/>
     </row>
-    <row r="214" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A214" s="75"/>
       <c r="E214" s="76"/>
       <c r="F214" s="23"/>
       <c r="G214" s="23"/>
     </row>
-    <row r="215" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A215" s="75"/>
       <c r="E215" s="76"/>
       <c r="F215" s="23"/>
       <c r="G215" s="23"/>
     </row>
-    <row r="216" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A216" s="75"/>
       <c r="E216" s="76"/>
       <c r="F216" s="23"/>
       <c r="G216" s="23"/>
     </row>
-    <row r="217" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A217" s="75"/>
       <c r="E217" s="76"/>
       <c r="F217" s="23"/>
       <c r="G217" s="23"/>
     </row>
-    <row r="218" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A218" s="75"/>
       <c r="E218" s="76"/>
       <c r="F218" s="23"/>
       <c r="G218" s="23"/>
     </row>
-    <row r="219" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A219" s="75"/>
       <c r="E219" s="76"/>
       <c r="F219" s="23"/>
       <c r="G219" s="23"/>
     </row>
-    <row r="220" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A220" s="75"/>
       <c r="E220" s="76"/>
       <c r="F220" s="23"/>
       <c r="G220" s="23"/>
     </row>
-    <row r="221" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A221" s="75"/>
       <c r="E221" s="76"/>
       <c r="F221" s="23"/>
       <c r="G221" s="23"/>
     </row>
-    <row r="222" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A222" s="75"/>
       <c r="E222" s="76"/>
       <c r="F222" s="23"/>
       <c r="G222" s="23"/>
     </row>
-    <row r="223" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A223" s="75"/>
       <c r="E223" s="76"/>
       <c r="F223" s="23"/>
       <c r="G223" s="23"/>
     </row>
-    <row r="224" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A224" s="75"/>
       <c r="E224" s="76"/>
       <c r="F224" s="23"/>
       <c r="G224" s="23"/>
     </row>
-    <row r="225" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A225" s="75"/>
       <c r="E225" s="76"/>
       <c r="F225" s="23"/>
       <c r="G225" s="23"/>
     </row>
-    <row r="226" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A226" s="75"/>
       <c r="E226" s="76"/>
       <c r="F226" s="23"/>
       <c r="G226" s="23"/>
     </row>
-    <row r="227" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A227" s="75"/>
       <c r="E227" s="76"/>
       <c r="F227" s="23"/>
       <c r="G227" s="23"/>
     </row>
-    <row r="228" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A228" s="75"/>
       <c r="E228" s="76"/>
       <c r="F228" s="23"/>
       <c r="G228" s="23"/>
     </row>
-    <row r="229" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A229" s="75"/>
       <c r="E229" s="76"/>
       <c r="F229" s="23"/>
       <c r="G229" s="23"/>
     </row>
-    <row r="230" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A230" s="75"/>
       <c r="E230" s="76"/>
       <c r="F230" s="23"/>
       <c r="G230" s="23"/>
     </row>
-    <row r="231" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A231" s="75"/>
       <c r="E231" s="76"/>
       <c r="F231" s="23"/>
       <c r="G231" s="23"/>
     </row>
-    <row r="232" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A232" s="75"/>
       <c r="E232" s="76"/>
       <c r="F232" s="23"/>
       <c r="G232" s="23"/>
     </row>
-    <row r="233" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A233" s="75"/>
       <c r="E233" s="76"/>
       <c r="F233" s="23"/>
       <c r="G233" s="23"/>
     </row>
-    <row r="234" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A234" s="75"/>
       <c r="E234" s="76"/>
       <c r="F234" s="23"/>
       <c r="G234" s="23"/>
     </row>
-    <row r="235" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A235" s="75"/>
       <c r="E235" s="76"/>
       <c r="F235" s="23"/>
       <c r="G235" s="23"/>
     </row>
-    <row r="236" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A236" s="75"/>
       <c r="E236" s="76"/>
       <c r="F236" s="23"/>
       <c r="G236" s="23"/>
     </row>
-    <row r="237" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A237" s="75"/>
       <c r="E237" s="76"/>
       <c r="F237" s="23"/>
       <c r="G237" s="23"/>
     </row>
-    <row r="238" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A238" s="75"/>
       <c r="E238" s="76"/>
       <c r="F238" s="23"/>
       <c r="G238" s="23"/>
     </row>
-    <row r="239" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A239" s="75"/>
       <c r="E239" s="76"/>
       <c r="F239" s="23"/>
       <c r="G239" s="23"/>
     </row>
-    <row r="240" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A240" s="75"/>
       <c r="E240" s="76"/>
       <c r="F240" s="23"/>
       <c r="G240" s="23"/>
     </row>
-    <row r="241" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A241" s="75"/>
       <c r="E241" s="76"/>
       <c r="F241" s="23"/>
       <c r="G241" s="23"/>
     </row>
-    <row r="242" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A242" s="75"/>
       <c r="E242" s="76"/>
       <c r="F242" s="23"/>
       <c r="G242" s="23"/>
     </row>
-    <row r="243" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A243" s="75"/>
       <c r="E243" s="76"/>
       <c r="F243" s="23"/>
       <c r="G243" s="23"/>
     </row>
-    <row r="244" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A244" s="75"/>
       <c r="E244" s="76"/>
       <c r="F244" s="23"/>
       <c r="G244" s="23"/>
     </row>
-    <row r="245" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A245" s="75"/>
       <c r="E245" s="76"/>
       <c r="F245" s="23"/>
       <c r="G245" s="23"/>
     </row>
-    <row r="246" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A246" s="75"/>
       <c r="E246" s="76"/>
       <c r="F246" s="23"/>
       <c r="G246" s="23"/>
     </row>
-    <row r="247" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A247" s="75"/>
       <c r="E247" s="76"/>
       <c r="F247" s="23"/>
       <c r="G247" s="23"/>
     </row>
-    <row r="248" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A248" s="75"/>
       <c r="E248" s="76"/>
       <c r="F248" s="23"/>
       <c r="G248" s="23"/>
     </row>
-    <row r="249" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A249" s="75"/>
       <c r="E249" s="76"/>
       <c r="F249" s="23"/>
       <c r="G249" s="23"/>
     </row>
-    <row r="250" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A250" s="75"/>
       <c r="E250" s="76"/>
       <c r="F250" s="23"/>
       <c r="G250" s="23"/>
     </row>
-    <row r="251" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A251" s="75"/>
       <c r="E251" s="76"/>
       <c r="F251" s="23"/>
       <c r="G251" s="23"/>
     </row>
-    <row r="252" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A252" s="75"/>
       <c r="E252" s="76"/>
       <c r="F252" s="23"/>
       <c r="G252" s="23"/>
     </row>
-    <row r="253" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A253" s="75"/>
       <c r="E253" s="76"/>
       <c r="F253" s="23"/>
       <c r="G253" s="23"/>
     </row>
-    <row r="254" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A254" s="75"/>
       <c r="E254" s="76"/>
       <c r="F254" s="23"/>
       <c r="G254" s="23"/>
     </row>
-    <row r="255" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A255" s="75"/>
       <c r="E255" s="76"/>
       <c r="F255" s="23"/>
       <c r="G255" s="23"/>
     </row>
-    <row r="256" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A256" s="75"/>
       <c r="E256" s="76"/>
       <c r="F256" s="23"/>
       <c r="G256" s="23"/>
     </row>
-    <row r="257" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A257" s="75"/>
       <c r="E257" s="76"/>
       <c r="F257" s="23"/>
       <c r="G257" s="23"/>
     </row>
-    <row r="258" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A258" s="75"/>
       <c r="E258" s="76"/>
       <c r="F258" s="23"/>
       <c r="G258" s="23"/>
     </row>
-    <row r="259" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A259" s="75"/>
       <c r="E259" s="76"/>
       <c r="F259" s="23"/>
       <c r="G259" s="23"/>
     </row>
-    <row r="260" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A260" s="75"/>
       <c r="E260" s="76"/>
       <c r="F260" s="23"/>
       <c r="G260" s="23"/>
     </row>
-    <row r="261" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A261" s="75"/>
       <c r="E261" s="76"/>
       <c r="F261" s="23"/>
       <c r="G261" s="23"/>
     </row>
-    <row r="262" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A262" s="75"/>
       <c r="E262" s="76"/>
       <c r="F262" s="23"/>
       <c r="G262" s="23"/>
     </row>
-    <row r="263" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A263" s="75"/>
       <c r="E263" s="76"/>
       <c r="F263" s="23"/>
       <c r="G263" s="23"/>
     </row>
-    <row r="264" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A264" s="75"/>
       <c r="E264" s="76"/>
       <c r="F264" s="23"/>
       <c r="G264" s="23"/>
     </row>
-    <row r="265" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A265" s="75"/>
       <c r="E265" s="76"/>
       <c r="F265" s="23"/>
       <c r="G265" s="23"/>
     </row>
-    <row r="266" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A266" s="75"/>
       <c r="E266" s="76"/>
       <c r="F266" s="23"/>
       <c r="G266" s="23"/>
     </row>
-    <row r="267" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A267" s="75"/>
       <c r="E267" s="76"/>
       <c r="F267" s="23"/>
       <c r="G267" s="23"/>
     </row>
-    <row r="268" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A268" s="75"/>
       <c r="E268" s="76"/>
       <c r="F268" s="23"/>
       <c r="G268" s="23"/>
     </row>
-    <row r="269" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A269" s="75"/>
       <c r="E269" s="76"/>
       <c r="F269" s="23"/>
       <c r="G269" s="23"/>
     </row>
-    <row r="270" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A270" s="75"/>
       <c r="E270" s="76"/>
       <c r="F270" s="23"/>
       <c r="G270" s="23"/>
     </row>
-    <row r="271" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A271" s="75"/>
       <c r="E271" s="76"/>
       <c r="F271" s="23"/>
       <c r="G271" s="23"/>
     </row>
-    <row r="272" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A272" s="75"/>
       <c r="E272" s="76"/>
       <c r="F272" s="23"/>
       <c r="G272" s="23"/>
     </row>
-    <row r="273" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A273" s="75"/>
       <c r="E273" s="76"/>
       <c r="F273" s="23"/>
       <c r="G273" s="23"/>
     </row>
-    <row r="274" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A274" s="75"/>
       <c r="E274" s="76"/>
       <c r="F274" s="23"/>
       <c r="G274" s="23"/>
     </row>
-    <row r="275" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A275" s="75"/>
       <c r="E275" s="76"/>
       <c r="F275" s="23"/>
       <c r="G275" s="23"/>
     </row>
-    <row r="276" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A276" s="75"/>
       <c r="E276" s="76"/>
       <c r="F276" s="23"/>
       <c r="G276" s="23"/>
     </row>
-    <row r="277" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A277" s="75"/>
       <c r="E277" s="76"/>
       <c r="F277" s="23"/>
       <c r="G277" s="23"/>
     </row>
-    <row r="278" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A278" s="75"/>
       <c r="E278" s="76"/>
       <c r="F278" s="23"/>
       <c r="G278" s="23"/>
     </row>
-    <row r="279" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A279" s="75"/>
       <c r="E279" s="76"/>
       <c r="F279" s="23"/>
       <c r="G279" s="23"/>
     </row>
-    <row r="280" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A280" s="75"/>
       <c r="E280" s="76"/>
       <c r="F280" s="23"/>
       <c r="G280" s="23"/>
     </row>
-    <row r="281" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A281" s="75"/>
       <c r="E281" s="76"/>
       <c r="F281" s="23"/>
       <c r="G281" s="23"/>
     </row>
-    <row r="282" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A282" s="75"/>
       <c r="E282" s="76"/>
       <c r="F282" s="23"/>
       <c r="G282" s="23"/>
     </row>
-    <row r="283" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A283" s="75"/>
       <c r="E283" s="76"/>
       <c r="F283" s="23"/>
       <c r="G283" s="23"/>
     </row>
-    <row r="284" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A284" s="75"/>
       <c r="E284" s="76"/>
       <c r="F284" s="23"/>
       <c r="G284" s="23"/>
     </row>
-    <row r="285" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A285" s="75"/>
       <c r="E285" s="76"/>
       <c r="F285" s="23"/>
       <c r="G285" s="23"/>
     </row>
-    <row r="286" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A286" s="75"/>
       <c r="E286" s="76"/>
       <c r="F286" s="23"/>
       <c r="G286" s="23"/>
     </row>
-    <row r="287" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A287" s="75"/>
       <c r="E287" s="76"/>
       <c r="F287" s="23"/>
       <c r="G287" s="23"/>
     </row>
-    <row r="288" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A288" s="75"/>
       <c r="E288" s="76"/>
       <c r="F288" s="23"/>
       <c r="G288" s="23"/>
     </row>
-    <row r="289" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A289" s="75"/>
       <c r="E289" s="76"/>
       <c r="F289" s="23"/>
       <c r="G289" s="23"/>
     </row>
-    <row r="290" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A290" s="75"/>
       <c r="E290" s="76"/>
       <c r="F290" s="23"/>
       <c r="G290" s="23"/>
     </row>
-    <row r="291" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A291" s="75"/>
       <c r="E291" s="76"/>
       <c r="F291" s="23"/>
       <c r="G291" s="23"/>
     </row>
-    <row r="292" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A292" s="75"/>
       <c r="E292" s="76"/>
       <c r="F292" s="23"/>
       <c r="G292" s="23"/>
     </row>
-    <row r="293" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A293" s="75"/>
       <c r="E293" s="76"/>
       <c r="F293" s="23"/>
       <c r="G293" s="23"/>
     </row>
-    <row r="294" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A294" s="75"/>
       <c r="E294" s="76"/>
       <c r="F294" s="23"/>
       <c r="G294" s="23"/>
     </row>
-    <row r="295" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A295" s="75"/>
       <c r="E295" s="76"/>
       <c r="F295" s="23"/>
       <c r="G295" s="23"/>
     </row>
-    <row r="296" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A296" s="75"/>
       <c r="E296" s="76"/>
       <c r="F296" s="23"/>
       <c r="G296" s="23"/>
     </row>
-    <row r="297" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A297" s="75"/>
       <c r="E297" s="76"/>
       <c r="F297" s="23"/>
       <c r="G297" s="23"/>
     </row>
-    <row r="298" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A298" s="75"/>
       <c r="E298" s="76"/>
       <c r="F298" s="23"/>
       <c r="G298" s="23"/>
     </row>
-    <row r="299" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A299" s="75"/>
       <c r="E299" s="76"/>
       <c r="F299" s="23"/>
       <c r="G299" s="23"/>
     </row>
-    <row r="300" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A300" s="75"/>
       <c r="E300" s="76"/>
       <c r="F300" s="23"/>
       <c r="G300" s="23"/>
     </row>
-    <row r="301" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A301" s="75"/>
       <c r="E301" s="76"/>
       <c r="F301" s="23"/>
       <c r="G301" s="23"/>
     </row>
-    <row r="302" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A302" s="75"/>
       <c r="E302" s="76"/>
       <c r="F302" s="23"/>
       <c r="G302" s="23"/>
     </row>
-    <row r="303" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A303" s="75"/>
       <c r="E303" s="76"/>
       <c r="F303" s="23"/>
       <c r="G303" s="23"/>
     </row>
-    <row r="304" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A304" s="75"/>
       <c r="E304" s="76"/>
       <c r="F304" s="23"/>
       <c r="G304" s="23"/>
     </row>
-    <row r="305" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A305" s="75"/>
       <c r="E305" s="76"/>
       <c r="F305" s="23"/>
       <c r="G305" s="23"/>
     </row>
-    <row r="306" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A306" s="75"/>
       <c r="E306" s="76"/>
       <c r="F306" s="23"/>
       <c r="G306" s="23"/>
     </row>
-    <row r="307" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A307" s="75"/>
       <c r="E307" s="76"/>
       <c r="F307" s="23"/>
       <c r="G307" s="23"/>
     </row>
-    <row r="308" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A308" s="75"/>
       <c r="E308" s="76"/>
       <c r="F308" s="23"/>
       <c r="G308" s="23"/>
     </row>
-    <row r="309" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A309" s="75"/>
       <c r="E309" s="76"/>
       <c r="F309" s="23"/>
       <c r="G309" s="23"/>
     </row>
-    <row r="310" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A310" s="75"/>
       <c r="E310" s="76"/>
       <c r="F310" s="23"/>
       <c r="G310" s="23"/>
     </row>
-    <row r="311" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A311" s="75"/>
       <c r="E311" s="76"/>
       <c r="F311" s="23"/>
       <c r="G311" s="23"/>
     </row>
-    <row r="312" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A312" s="75"/>
       <c r="E312" s="76"/>
       <c r="F312" s="23"/>
       <c r="G312" s="23"/>
     </row>
-    <row r="313" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A313" s="75"/>
       <c r="E313" s="76"/>
       <c r="F313" s="23"/>
       <c r="G313" s="23"/>
     </row>
-    <row r="314" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A314" s="75"/>
       <c r="E314" s="76"/>
       <c r="F314" s="23"/>
       <c r="G314" s="23"/>
     </row>
-    <row r="315" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A315" s="75"/>
       <c r="E315" s="76"/>
       <c r="F315" s="23"/>
       <c r="G315" s="23"/>
     </row>
-    <row r="316" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A316" s="75"/>
       <c r="E316" s="76"/>
       <c r="F316" s="23"/>
       <c r="G316" s="23"/>
     </row>
-    <row r="317" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A317" s="75"/>
       <c r="E317" s="76"/>
       <c r="F317" s="23"/>
       <c r="G317" s="23"/>
     </row>
-    <row r="318" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A318" s="75"/>
       <c r="E318" s="76"/>
       <c r="F318" s="23"/>
       <c r="G318" s="23"/>
     </row>
-    <row r="319" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A319" s="75"/>
       <c r="E319" s="76"/>
       <c r="F319" s="23"/>
       <c r="G319" s="23"/>
     </row>
-    <row r="320" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A320" s="75"/>
       <c r="E320" s="76"/>
       <c r="F320" s="23"/>
       <c r="G320" s="23"/>
     </row>
-    <row r="321" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A321" s="75"/>
       <c r="E321" s="76"/>
       <c r="F321" s="23"/>
       <c r="G321" s="23"/>
     </row>
-    <row r="322" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A322" s="75"/>
       <c r="E322" s="76"/>
       <c r="F322" s="23"/>
       <c r="G322" s="23"/>
     </row>
-    <row r="323" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A323" s="75"/>
       <c r="E323" s="76"/>
       <c r="F323" s="23"/>
       <c r="G323" s="23"/>
     </row>
-    <row r="324" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A324" s="75"/>
       <c r="E324" s="76"/>
       <c r="F324" s="23"/>
       <c r="G324" s="23"/>
     </row>
-    <row r="325" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A325" s="75"/>
       <c r="E325" s="76"/>
       <c r="F325" s="23"/>
       <c r="G325" s="23"/>
     </row>
-    <row r="326" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A326" s="75"/>
       <c r="E326" s="76"/>
       <c r="F326" s="23"/>
       <c r="G326" s="23"/>
     </row>
-    <row r="327" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A327" s="75"/>
       <c r="E327" s="76"/>
       <c r="F327" s="23"/>
       <c r="G327" s="23"/>
     </row>
-    <row r="328" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A328" s="75"/>
       <c r="E328" s="76"/>
       <c r="F328" s="23"/>
       <c r="G328" s="23"/>
     </row>
-    <row r="329" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A329" s="75"/>
       <c r="E329" s="76"/>
       <c r="F329" s="23"/>
       <c r="G329" s="23"/>
     </row>
-    <row r="330" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A330" s="75"/>
       <c r="E330" s="76"/>
       <c r="F330" s="23"/>
       <c r="G330" s="23"/>
     </row>
-    <row r="331" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A331" s="75"/>
       <c r="E331" s="76"/>
       <c r="F331" s="23"/>
       <c r="G331" s="23"/>
     </row>
-    <row r="332" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A332" s="75"/>
       <c r="E332" s="76"/>
       <c r="F332" s="23"/>
       <c r="G332" s="23"/>
     </row>
-    <row r="333" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A333" s="75"/>
       <c r="E333" s="76"/>
       <c r="F333" s="23"/>
       <c r="G333" s="23"/>
     </row>
-    <row r="334" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A334" s="75"/>
       <c r="E334" s="76"/>
       <c r="F334" s="23"/>
       <c r="G334" s="23"/>
     </row>
-    <row r="335" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A335" s="75"/>
       <c r="E335" s="76"/>
       <c r="F335" s="23"/>
       <c r="G335" s="23"/>
     </row>
-    <row r="336" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A336" s="75"/>
       <c r="E336" s="76"/>
       <c r="F336" s="23"/>
       <c r="G336" s="23"/>
     </row>
-    <row r="337" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A337" s="75"/>
       <c r="E337" s="76"/>
       <c r="F337" s="23"/>
       <c r="G337" s="23"/>
     </row>
-    <row r="338" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A338" s="75"/>
       <c r="E338" s="76"/>
       <c r="F338" s="23"/>
       <c r="G338" s="23"/>
     </row>
-    <row r="339" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A339" s="75"/>
       <c r="E339" s="76"/>
       <c r="F339" s="23"/>
       <c r="G339" s="23"/>
     </row>
-    <row r="340" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A340" s="75"/>
       <c r="E340" s="76"/>
       <c r="F340" s="23"/>
       <c r="G340" s="23"/>
     </row>
-    <row r="341" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A341" s="75"/>
       <c r="E341" s="76"/>
       <c r="F341" s="23"/>
       <c r="G341" s="23"/>
     </row>
-    <row r="342" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A342" s="75"/>
       <c r="E342" s="76"/>
       <c r="F342" s="23"/>
       <c r="G342" s="23"/>
     </row>
-    <row r="343" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A343" s="75"/>
       <c r="E343" s="76"/>
       <c r="F343" s="23"/>
       <c r="G343" s="23"/>
     </row>
-    <row r="344" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A344" s="75"/>
       <c r="E344" s="76"/>
       <c r="F344" s="23"/>
       <c r="G344" s="23"/>
     </row>
-    <row r="345" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A345" s="75"/>
       <c r="E345" s="76"/>
       <c r="F345" s="23"/>
       <c r="G345" s="23"/>
     </row>
-    <row r="346" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A346" s="75"/>
       <c r="E346" s="76"/>
       <c r="F346" s="23"/>
       <c r="G346" s="23"/>
     </row>
-    <row r="347" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A347" s="75"/>
       <c r="E347" s="76"/>
       <c r="F347" s="23"/>
       <c r="G347" s="23"/>
     </row>
-    <row r="348" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A348" s="75"/>
       <c r="E348" s="76"/>
       <c r="F348" s="23"/>
       <c r="G348" s="23"/>
     </row>
-    <row r="349" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A349" s="75"/>
       <c r="E349" s="76"/>
       <c r="F349" s="23"/>
       <c r="G349" s="23"/>
     </row>
-    <row r="350" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A350" s="75"/>
       <c r="E350" s="76"/>
       <c r="F350" s="23"/>
       <c r="G350" s="23"/>
     </row>
-    <row r="351" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A351" s="75"/>
       <c r="E351" s="76"/>
       <c r="F351" s="23"/>
       <c r="G351" s="23"/>
     </row>
-    <row r="352" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A352" s="75"/>
       <c r="E352" s="76"/>
       <c r="F352" s="23"/>
       <c r="G352" s="23"/>
     </row>
-    <row r="353" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A353" s="75"/>
       <c r="E353" s="76"/>
       <c r="F353" s="23"/>
       <c r="G353" s="23"/>
     </row>
-    <row r="354" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A354" s="75"/>
       <c r="E354" s="76"/>
       <c r="F354" s="23"/>
       <c r="G354" s="23"/>
     </row>
-    <row r="355" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A355" s="75"/>
       <c r="E355" s="76"/>
       <c r="F355" s="23"/>
       <c r="G355" s="23"/>
     </row>
-    <row r="356" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A356" s="75"/>
       <c r="E356" s="76"/>
       <c r="F356" s="23"/>
       <c r="G356" s="23"/>
     </row>
-    <row r="357" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A357" s="75"/>
       <c r="E357" s="76"/>
       <c r="F357" s="23"/>
       <c r="G357" s="23"/>
     </row>
-    <row r="358" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A358" s="75"/>
       <c r="E358" s="76"/>
       <c r="F358" s="23"/>
       <c r="G358" s="23"/>
     </row>
-    <row r="359" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A359" s="75"/>
       <c r="E359" s="76"/>
       <c r="F359" s="23"/>
       <c r="G359" s="23"/>
     </row>
-    <row r="360" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A360" s="75"/>
       <c r="E360" s="76"/>
       <c r="F360" s="23"/>
       <c r="G360" s="23"/>
     </row>
-    <row r="361" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A361" s="75"/>
       <c r="E361" s="76"/>
       <c r="F361" s="23"/>
       <c r="G361" s="23"/>
     </row>
-    <row r="362" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A362" s="75"/>
       <c r="E362" s="76"/>
       <c r="F362" s="23"/>
       <c r="G362" s="23"/>
     </row>
-    <row r="363" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A363" s="75"/>
       <c r="E363" s="76"/>
       <c r="F363" s="23"/>
       <c r="G363" s="23"/>
     </row>
-    <row r="364" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A364" s="75"/>
       <c r="E364" s="76"/>
       <c r="F364" s="23"/>
       <c r="G364" s="23"/>
     </row>
-    <row r="365" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A365" s="75"/>
       <c r="E365" s="76"/>
       <c r="F365" s="23"/>
       <c r="G365" s="23"/>
     </row>
-    <row r="366" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A366" s="75"/>
       <c r="E366" s="76"/>
       <c r="F366" s="23"/>
       <c r="G366" s="23"/>
     </row>
-    <row r="367" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A367" s="75"/>
       <c r="E367" s="76"/>
       <c r="F367" s="23"/>
       <c r="G367" s="23"/>
     </row>
-    <row r="368" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A368" s="75"/>
       <c r="E368" s="76"/>
       <c r="F368" s="23"/>
       <c r="G368" s="23"/>
     </row>
-    <row r="369" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A369" s="75"/>
       <c r="E369" s="76"/>
       <c r="F369" s="23"/>
       <c r="G369" s="23"/>
     </row>
-    <row r="370" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A370" s="75"/>
       <c r="E370" s="76"/>
       <c r="F370" s="23"/>
       <c r="G370" s="23"/>
     </row>
-    <row r="371" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A371" s="75"/>
       <c r="E371" s="76"/>
       <c r="F371" s="23"/>
       <c r="G371" s="23"/>
     </row>
-    <row r="372" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A372" s="75"/>
       <c r="E372" s="76"/>
       <c r="F372" s="23"/>
       <c r="G372" s="23"/>
     </row>
-    <row r="373" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A373" s="75"/>
       <c r="E373" s="76"/>
       <c r="F373" s="23"/>
       <c r="G373" s="23"/>
     </row>
-    <row r="374" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A374" s="75"/>
       <c r="E374" s="76"/>
       <c r="F374" s="23"/>
       <c r="G374" s="23"/>
     </row>
-    <row r="375" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A375" s="75"/>
       <c r="E375" s="76"/>
       <c r="F375" s="23"/>
       <c r="G375" s="23"/>
     </row>
-    <row r="376" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A376" s="75"/>
       <c r="E376" s="76"/>
       <c r="F376" s="23"/>
       <c r="G376" s="23"/>
     </row>
-    <row r="377" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A377" s="75"/>
       <c r="E377" s="76"/>
       <c r="F377" s="23"/>
       <c r="G377" s="23"/>
     </row>
-    <row r="378" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A378" s="75"/>
       <c r="E378" s="76"/>
       <c r="F378" s="23"/>
       <c r="G378" s="23"/>
     </row>
-    <row r="379" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A379" s="75"/>
       <c r="E379" s="76"/>
       <c r="F379" s="23"/>
       <c r="G379" s="23"/>
     </row>
-    <row r="380" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A380" s="75"/>
       <c r="E380" s="76"/>
       <c r="F380" s="23"/>
       <c r="G380" s="23"/>
     </row>
-    <row r="381" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A381" s="75"/>
       <c r="E381" s="76"/>
       <c r="F381" s="23"/>
       <c r="G381" s="23"/>
     </row>
-    <row r="382" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A382" s="75"/>
       <c r="E382" s="76"/>
       <c r="F382" s="23"/>
       <c r="G382" s="23"/>
     </row>
-    <row r="383" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A383" s="75"/>
       <c r="E383" s="76"/>
       <c r="F383" s="23"/>
       <c r="G383" s="23"/>
     </row>
-    <row r="384" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A384" s="75"/>
       <c r="E384" s="76"/>
       <c r="F384" s="23"/>
       <c r="G384" s="23"/>
     </row>
-    <row r="385" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="385" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A385" s="75"/>
       <c r="E385" s="76"/>
       <c r="F385" s="23"/>
       <c r="G385" s="23"/>
     </row>
-    <row r="386" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="386" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A386" s="75"/>
       <c r="E386" s="76"/>
       <c r="F386" s="23"/>
       <c r="G386" s="23"/>
     </row>
-    <row r="387" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="387" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A387" s="75"/>
       <c r="E387" s="76"/>
       <c r="F387" s="23"/>
       <c r="G387" s="23"/>
     </row>
-    <row r="388" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="388" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A388" s="75"/>
       <c r="E388" s="76"/>
       <c r="F388" s="23"/>
       <c r="G388" s="23"/>
     </row>
-    <row r="389" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A389" s="75"/>
       <c r="E389" s="76"/>
       <c r="F389" s="23"/>
       <c r="G389" s="23"/>
     </row>
-    <row r="390" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="390" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A390" s="75"/>
       <c r="E390" s="76"/>
       <c r="F390" s="23"/>
       <c r="G390" s="23"/>
     </row>
-    <row r="391" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="391" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A391" s="75"/>
       <c r="E391" s="76"/>
       <c r="F391" s="23"/>
       <c r="G391" s="23"/>
     </row>
-    <row r="392" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A392" s="75"/>
       <c r="E392" s="76"/>
       <c r="F392" s="23"/>
       <c r="G392" s="23"/>
     </row>
-    <row r="393" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="393" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A393" s="75"/>
       <c r="E393" s="76"/>
       <c r="F393" s="23"/>
       <c r="G393" s="23"/>
     </row>
-    <row r="394" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A394" s="75"/>
       <c r="E394" s="76"/>
       <c r="F394" s="23"/>
       <c r="G394" s="23"/>
     </row>
-    <row r="395" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A395" s="75"/>
       <c r="E395" s="76"/>
       <c r="F395" s="23"/>
       <c r="G395" s="23"/>
     </row>
-    <row r="396" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A396" s="75"/>
       <c r="E396" s="76"/>
       <c r="F396" s="23"/>
       <c r="G396" s="23"/>
     </row>
-    <row r="397" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A397" s="75"/>
       <c r="E397" s="76"/>
       <c r="F397" s="23"/>
       <c r="G397" s="23"/>
     </row>
-    <row r="398" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A398" s="75"/>
       <c r="E398" s="76"/>
       <c r="F398" s="23"/>
       <c r="G398" s="23"/>
     </row>
-    <row r="399" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A399" s="75"/>
       <c r="E399" s="76"/>
       <c r="F399" s="23"/>
       <c r="G399" s="23"/>
     </row>
-    <row r="400" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="400" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A400" s="75"/>
       <c r="E400" s="76"/>
       <c r="F400" s="23"/>
       <c r="G400" s="23"/>
     </row>
-    <row r="401" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="401" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A401" s="75"/>
       <c r="E401" s="76"/>
       <c r="F401" s="23"/>
       <c r="G401" s="23"/>
     </row>
-    <row r="402" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="402" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A402" s="75"/>
       <c r="E402" s="76"/>
       <c r="F402" s="23"/>
       <c r="G402" s="23"/>
     </row>
-    <row r="403" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="403" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A403" s="75"/>
       <c r="E403" s="76"/>
       <c r="F403" s="23"/>
       <c r="G403" s="23"/>
     </row>
-    <row r="404" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="404" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A404" s="75"/>
       <c r="E404" s="76"/>
       <c r="F404" s="23"/>
       <c r="G404" s="23"/>
     </row>
-    <row r="405" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="405" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A405" s="75"/>
       <c r="E405" s="76"/>
       <c r="F405" s="23"/>
       <c r="G405" s="23"/>
     </row>
-    <row r="406" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="406" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A406" s="75"/>
       <c r="E406" s="76"/>
       <c r="F406" s="23"/>
       <c r="G406" s="23"/>
     </row>
-    <row r="407" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="407" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A407" s="75"/>
       <c r="E407" s="76"/>
       <c r="F407" s="23"/>
       <c r="G407" s="23"/>
     </row>
-    <row r="408" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="408" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A408" s="75"/>
       <c r="E408" s="76"/>
       <c r="F408" s="23"/>
       <c r="G408" s="23"/>
     </row>
-    <row r="409" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="409" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A409" s="75"/>
       <c r="E409" s="76"/>
       <c r="F409" s="23"/>
       <c r="G409" s="23"/>
     </row>
-    <row r="410" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="410" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A410" s="75"/>
       <c r="E410" s="76"/>
       <c r="F410" s="23"/>
       <c r="G410" s="23"/>
     </row>
-    <row r="411" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="411" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A411" s="75"/>
       <c r="E411" s="76"/>
       <c r="F411" s="23"/>
       <c r="G411" s="23"/>
     </row>
-    <row r="412" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="412" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A412" s="75"/>
       <c r="E412" s="76"/>
       <c r="F412" s="23"/>
       <c r="G412" s="23"/>
     </row>
-    <row r="413" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="413" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A413" s="75"/>
       <c r="E413" s="76"/>
       <c r="F413" s="23"/>
       <c r="G413" s="23"/>
     </row>
-    <row r="414" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="414" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A414" s="75"/>
       <c r="E414" s="76"/>
       <c r="F414" s="23"/>
       <c r="G414" s="23"/>
     </row>
-    <row r="415" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="415" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A415" s="75"/>
       <c r="E415" s="76"/>
       <c r="F415" s="23"/>
       <c r="G415" s="23"/>
     </row>
-    <row r="416" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="416" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A416" s="75"/>
       <c r="E416" s="76"/>
       <c r="F416" s="23"/>
       <c r="G416" s="23"/>
     </row>
-    <row r="417" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="417" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A417" s="75"/>
       <c r="E417" s="76"/>
       <c r="F417" s="23"/>
       <c r="G417" s="23"/>
     </row>
-    <row r="418" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="418" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A418" s="75"/>
       <c r="E418" s="76"/>
       <c r="F418" s="23"/>
       <c r="G418" s="23"/>
     </row>
-    <row r="419" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="419" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A419" s="75"/>
       <c r="E419" s="76"/>
       <c r="F419" s="23"/>
       <c r="G419" s="23"/>
     </row>
-    <row r="420" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="420" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A420" s="75"/>
       <c r="E420" s="76"/>
       <c r="F420" s="23"/>
       <c r="G420" s="23"/>
     </row>
-    <row r="421" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="421" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A421" s="75"/>
       <c r="E421" s="76"/>
       <c r="F421" s="23"/>
       <c r="G421" s="23"/>
     </row>
-    <row r="422" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="422" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A422" s="75"/>
       <c r="E422" s="76"/>
       <c r="F422" s="23"/>
       <c r="G422" s="23"/>
     </row>
-    <row r="423" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="423" spans="1:7" s="24" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A423" s="75"/>
       <c r="E423" s="76"/>
       <c r="F423" s="23"/>

</xml_diff>